<commit_message>
Sprint 5 Day 31: Cash Flow Intelligence Module completed
</commit_message>
<xml_diff>
--- a/output/cashflow_intelligence.xlsx
+++ b/output/cashflow_intelligence.xlsx
@@ -485,7 +485,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>3.22</v>
+        <v>2.43</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -504,7 +504,7 @@
         <v>15.97680185259178</v>
       </c>
       <c r="H2" t="n">
-        <v>469.8832684824903</v>
+        <v>502.7477102414655</v>
       </c>
       <c r="I2" t="b">
         <v>0</v>
@@ -547,7 +547,7 @@
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="n">
-        <v>1025.127334465195</v>
+        <v>504.8494983277591</v>
       </c>
       <c r="I3" t="b">
         <v>0</v>
@@ -590,7 +590,7 @@
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="n">
-        <v>169.4380545514295</v>
+        <v>309.2053973013493</v>
       </c>
       <c r="I4" t="b">
         <v>0</v>
@@ -633,7 +633,7 @@
       </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="n">
-        <v>400.0518672199171</v>
+        <v>612.1428571428571</v>
       </c>
       <c r="I5" t="b">
         <v>0</v>
@@ -676,7 +676,7 @@
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="n">
-        <v>154.1414348763215</v>
+        <v>185.3158933859822</v>
       </c>
       <c r="I6" t="b">
         <v>0</v>
@@ -719,7 +719,7 @@
       </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="n">
-        <v>111.6979347311998</v>
+        <v>68.03015027125642</v>
       </c>
       <c r="I7" t="b">
         <v>0</v>
@@ -729,7 +729,7 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>Average</t>
         </is>
       </c>
     </row>
@@ -745,7 +745,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>1.47</v>
+        <v>1.22</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -762,7 +762,7 @@
       </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="n">
-        <v>145.8537845517954</v>
+        <v>119.1642043056142</v>
       </c>
       <c r="I8" t="b">
         <v>0</v>
@@ -805,7 +805,7 @@
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="n">
-        <v>156.8627450980392</v>
+        <v>205.3475935828877</v>
       </c>
       <c r="I9" t="b">
         <v>0</v>
@@ -850,7 +850,7 @@
         <v>15.56823256217168</v>
       </c>
       <c r="H10" t="n">
-        <v>131.8073850140358</v>
+        <v>109.823677581864</v>
       </c>
       <c r="I10" t="b">
         <v>0</v>
@@ -936,7 +936,7 @@
       </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="n">
-        <v>-21.05283104676722</v>
+        <v>-22.34423394071035</v>
       </c>
       <c r="I12" t="b">
         <v>1</v>
@@ -981,7 +981,7 @@
         <v>9.385229927877292</v>
       </c>
       <c r="H13" t="n">
-        <v>88.97028897028896</v>
+        <v>85.0804359107421</v>
       </c>
       <c r="I13" t="b">
         <v>0</v>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="n">
-        <v>-415.7021791767554</v>
+        <v>-440.3590894517474</v>
       </c>
       <c r="I14" t="b">
         <v>1</v>
@@ -1069,7 +1069,7 @@
         <v>27.2167818274256</v>
       </c>
       <c r="H15" t="n">
-        <v>25.92839967940155</v>
+        <v>26.35437881873727</v>
       </c>
       <c r="I15" t="b">
         <v>0</v>
@@ -1112,7 +1112,7 @@
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="n">
-        <v>-472.8052505036064</v>
+        <v>-503.4945678499758</v>
       </c>
       <c r="I16" t="b">
         <v>1</v>
@@ -1155,7 +1155,7 @@
       </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="n">
-        <v>-31.14575059571088</v>
+        <v>-33.25030473263024</v>
       </c>
       <c r="I17" t="b">
         <v>1</v>
@@ -1198,7 +1198,7 @@
       </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="n">
-        <v>102.5985465756441</v>
+        <v>116.9134253450439</v>
       </c>
       <c r="I18" t="b">
         <v>0</v>
@@ -1243,7 +1243,7 @@
         <v>19.46310700548934</v>
       </c>
       <c r="H19" t="n">
-        <v>571.0625361899247</v>
+        <v>921.9210095816779</v>
       </c>
       <c r="I19" t="b">
         <v>0</v>
@@ -1286,7 +1286,7 @@
       </c>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="n">
-        <v>-834.3820224719101</v>
+        <v>-1316.666666666667</v>
       </c>
       <c r="I20" t="b">
         <v>1</v>
@@ -1331,7 +1331,7 @@
         <v>37.29762744346468</v>
       </c>
       <c r="H21" t="n">
-        <v>60.12476007677543</v>
+        <v>50.32128514056225</v>
       </c>
       <c r="I21" t="b">
         <v>0</v>
@@ -1376,7 +1376,7 @@
         <v>24.30118345247379</v>
       </c>
       <c r="H22" t="n">
-        <v>261.6572011067424</v>
+        <v>133.7950035369894</v>
       </c>
       <c r="I22" t="b">
         <v>0</v>
@@ -1421,7 +1421,7 @@
         <v>21.81530931380111</v>
       </c>
       <c r="H23" t="n">
-        <v>120.8548614372945</v>
+        <v>120.5716963448922</v>
       </c>
       <c r="I23" t="b">
         <v>0</v>
@@ -1466,7 +1466,7 @@
         <v>5.247691552181655</v>
       </c>
       <c r="H24" t="n">
-        <v>90.79717578902903</v>
+        <v>97.6949548730602</v>
       </c>
       <c r="I24" t="b">
         <v>0</v>
@@ -1509,7 +1509,7 @@
       </c>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="n">
-        <v>-926.34994807892</v>
+        <v>-1043.362573099415</v>
       </c>
       <c r="I25" t="b">
         <v>1</v>
@@ -1552,7 +1552,7 @@
       </c>
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="n">
-        <v>82.89552837377181</v>
+        <v>99.51853635050554</v>
       </c>
       <c r="I26" t="b">
         <v>0</v>
@@ -1597,7 +1597,7 @@
         <v>5.863057152249307</v>
       </c>
       <c r="H27" t="n">
-        <v>52.70160116448326</v>
+        <v>48.44389734806926</v>
       </c>
       <c r="I27" t="b">
         <v>0</v>
@@ -1642,7 +1642,7 @@
         <v>13.93946746062713</v>
       </c>
       <c r="H28" t="n">
-        <v>114.375</v>
+        <v>111.1540585311982</v>
       </c>
       <c r="I28" t="b">
         <v>0</v>
@@ -1687,7 +1687,7 @@
         <v>14.43934874408408</v>
       </c>
       <c r="H29" t="n">
-        <v>68.68191721132898</v>
+        <v>78.8125</v>
       </c>
       <c r="I29" t="b">
         <v>0</v>
@@ -1732,7 +1732,7 @@
         <v>-11.76910917974342</v>
       </c>
       <c r="H30" t="n">
-        <v>63.41158841158842</v>
+        <v>93.20851688693098</v>
       </c>
       <c r="I30" t="b">
         <v>0</v>
@@ -1775,7 +1775,7 @@
       </c>
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="n">
-        <v>100.9558823529412</v>
+        <v>108.2807570977918</v>
       </c>
       <c r="I31" t="b">
         <v>0</v>
@@ -1818,7 +1818,7 @@
       </c>
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="n">
-        <v>83.38839941262849</v>
+        <v>81.44496235209753</v>
       </c>
       <c r="I32" t="b">
         <v>0</v>
@@ -1861,7 +1861,7 @@
       </c>
       <c r="G33" t="inlineStr"/>
       <c r="H33" t="n">
-        <v>87.25398313027179</v>
+        <v>93.07673081729567</v>
       </c>
       <c r="I33" t="b">
         <v>0</v>
@@ -1904,7 +1904,7 @@
       </c>
       <c r="G34" t="inlineStr"/>
       <c r="H34" t="n">
-        <v>109.0546746382463</v>
+        <v>127.0928001615672</v>
       </c>
       <c r="I34" t="b">
         <v>0</v>
@@ -1947,7 +1947,7 @@
       </c>
       <c r="G35" t="inlineStr"/>
       <c r="H35" t="n">
-        <v>-456.9536423841059</v>
+        <v>-368.9839572192514</v>
       </c>
       <c r="I35" t="b">
         <v>0</v>
@@ -1990,7 +1990,7 @@
       </c>
       <c r="G36" t="inlineStr"/>
       <c r="H36" t="n">
-        <v>-123.3061083630507</v>
+        <v>-107.989119484183</v>
       </c>
       <c r="I36" t="b">
         <v>1</v>
@@ -2035,7 +2035,7 @@
         <v>-5.002096841865733</v>
       </c>
       <c r="H37" t="n">
-        <v>97.09631728045326</v>
+        <v>108.3080974325214</v>
       </c>
       <c r="I37" t="b">
         <v>0</v>
@@ -2080,7 +2080,7 @@
         <v>-3.469343496883137</v>
       </c>
       <c r="H38" t="n">
-        <v>139.5</v>
+        <v>153.6585365853659</v>
       </c>
       <c r="I38" t="b">
         <v>0</v>
@@ -2125,7 +2125,7 @@
         <v>20.00447181280611</v>
       </c>
       <c r="H39" t="n">
-        <v>131.3901082821188</v>
+        <v>142.8898790579249</v>
       </c>
       <c r="I39" t="b">
         <v>0</v>
@@ -2168,7 +2168,7 @@
       </c>
       <c r="G40" t="inlineStr"/>
       <c r="H40" t="n">
-        <v>26.42306839596497</v>
+        <v>29.13699844146319</v>
       </c>
       <c r="I40" t="b">
         <v>0</v>
@@ -2211,7 +2211,7 @@
       </c>
       <c r="G41" t="inlineStr"/>
       <c r="H41" t="n">
-        <v>613.6805953062392</v>
+        <v>681.1308767471411</v>
       </c>
       <c r="I41" t="b">
         <v>0</v>
@@ -2256,7 +2256,7 @@
         <v>8.674914145052593</v>
       </c>
       <c r="H42" t="n">
-        <v>119.1144447132833</v>
+        <v>131.560662747194</v>
       </c>
       <c r="I42" t="b">
         <v>0</v>
@@ -2299,7 +2299,7 @@
       </c>
       <c r="G43" t="inlineStr"/>
       <c r="H43" t="n">
-        <v>192.6329276105061</v>
+        <v>236.8882323978336</v>
       </c>
       <c r="I43" t="b">
         <v>0</v>
@@ -2344,7 +2344,7 @@
         <v>9.689663003888427</v>
       </c>
       <c r="H44" t="n">
-        <v>143.8040345821325</v>
+        <v>150.4473837774752</v>
       </c>
       <c r="I44" t="b">
         <v>0</v>
@@ -2387,7 +2387,7 @@
       </c>
       <c r="G45" t="inlineStr"/>
       <c r="H45" t="n">
-        <v>300.0686813186813</v>
+        <v>341.3207178663657</v>
       </c>
       <c r="I45" t="b">
         <v>0</v>
@@ -2432,7 +2432,7 @@
         <v>32.49553261764786</v>
       </c>
       <c r="H46" t="n">
-        <v>95.59173947577443</v>
+        <v>125.4299114121939</v>
       </c>
       <c r="I46" t="b">
         <v>0</v>
@@ -2475,7 +2475,7 @@
       </c>
       <c r="G47" t="inlineStr"/>
       <c r="H47" t="n">
-        <v>-751.0266940451745</v>
+        <v>-859.5769682726205</v>
       </c>
       <c r="I47" t="b">
         <v>0</v>
@@ -2518,7 +2518,7 @@
       </c>
       <c r="G48" t="inlineStr"/>
       <c r="H48" t="n">
-        <v>348.7487652288443</v>
+        <v>259.3730868127832</v>
       </c>
       <c r="I48" t="b">
         <v>0</v>
@@ -2561,7 +2561,7 @@
       </c>
       <c r="G49" t="inlineStr"/>
       <c r="H49" t="n">
-        <v>-207.3750307805959</v>
+        <v>-188.1899441340782</v>
       </c>
       <c r="I49" t="b">
         <v>0</v>
@@ -2606,7 +2606,7 @@
         <v>14.69779172398365</v>
       </c>
       <c r="H50" t="n">
-        <v>91.05356304402788</v>
+        <v>96.04541298384639</v>
       </c>
       <c r="I50" t="b">
         <v>0</v>
@@ -2651,7 +2651,7 @@
         <v>84.86188044662759</v>
       </c>
       <c r="H51" t="n">
-        <v>651.7462645522046</v>
+        <v>164.7297328606844</v>
       </c>
       <c r="I51" t="b">
         <v>0</v>
@@ -2696,7 +2696,7 @@
         <v>45.37464474156747</v>
       </c>
       <c r="H52" t="n">
-        <v>73.5</v>
+        <v>79.38793879387939</v>
       </c>
       <c r="I52" t="b">
         <v>0</v>
@@ -2739,7 +2739,7 @@
       </c>
       <c r="G53" t="inlineStr"/>
       <c r="H53" t="n">
-        <v>121.0647085819183</v>
+        <v>123.4248284466625</v>
       </c>
       <c r="I53" t="b">
         <v>0</v>
@@ -2784,7 +2784,7 @@
         <v>17.36255738803865</v>
       </c>
       <c r="H54" t="n">
-        <v>82.47635508185702</v>
+        <v>82.78637174112092</v>
       </c>
       <c r="I54" t="b">
         <v>0</v>
@@ -2827,7 +2827,7 @@
       </c>
       <c r="G55" t="inlineStr"/>
       <c r="H55" t="n">
-        <v>118.7351778656127</v>
+        <v>101.0937237085647</v>
       </c>
       <c r="I55" t="b">
         <v>0</v>
@@ -2872,7 +2872,7 @@
         <v>-19.25925925925925</v>
       </c>
       <c r="H56" t="n">
-        <v>-42.19041692594897</v>
+        <v>-42.24299065420561</v>
       </c>
       <c r="I56" t="b">
         <v>0</v>
@@ -2915,7 +2915,7 @@
       </c>
       <c r="G57" t="inlineStr"/>
       <c r="H57" t="n">
-        <v>313.5814889336016</v>
+        <v>361.3913043478261</v>
       </c>
       <c r="I57" t="b">
         <v>0</v>
@@ -2958,7 +2958,7 @@
       </c>
       <c r="G58" t="inlineStr"/>
       <c r="H58" t="n">
-        <v>364.6739130434783</v>
+        <v>134.6038114343029</v>
       </c>
       <c r="I58" t="b">
         <v>0</v>
@@ -3001,7 +3001,7 @@
       </c>
       <c r="G59" t="inlineStr"/>
       <c r="H59" t="n">
-        <v>69.61828672880603</v>
+        <v>86.11980453522209</v>
       </c>
       <c r="I59" t="b">
         <v>0</v>
@@ -3011,7 +3011,7 @@
       </c>
       <c r="K59" t="inlineStr">
         <is>
-          <t>Average</t>
+          <t>Good</t>
         </is>
       </c>
     </row>
@@ -3046,7 +3046,7 @@
         <v>-48.21728841371581</v>
       </c>
       <c r="H60" t="n">
-        <v>62.99315134561589</v>
+        <v>63.84299540522045</v>
       </c>
       <c r="I60" t="b">
         <v>0</v>
@@ -3089,7 +3089,7 @@
       </c>
       <c r="G61" t="inlineStr"/>
       <c r="H61" t="n">
-        <v>100.0398247710076</v>
+        <v>161.6473616473616</v>
       </c>
       <c r="I61" t="b">
         <v>0</v>
@@ -3132,7 +3132,7 @@
       </c>
       <c r="G62" t="inlineStr"/>
       <c r="H62" t="n">
-        <v>113.1021671826626</v>
+        <v>117.4889046118222</v>
       </c>
       <c r="I62" t="b">
         <v>0</v>
@@ -3177,7 +3177,7 @@
         <v>14.79620583960055</v>
       </c>
       <c r="H63" t="n">
-        <v>123.9615216440752</v>
+        <v>123.6641221374046</v>
       </c>
       <c r="I63" t="b">
         <v>0</v>
@@ -3220,7 +3220,7 @@
       </c>
       <c r="G64" t="inlineStr"/>
       <c r="H64" t="n">
-        <v>-43.27773080175263</v>
+        <v>-45.8842705786471</v>
       </c>
       <c r="I64" t="b">
         <v>1</v>
@@ -3265,7 +3265,7 @@
         <v>16.27250444793893</v>
       </c>
       <c r="H65" t="n">
-        <v>119.8274017545111</v>
+        <v>124.5625741399763</v>
       </c>
       <c r="I65" t="b">
         <v>0</v>
@@ -3310,7 +3310,7 @@
         <v>7.992990088177754</v>
       </c>
       <c r="H66" t="n">
-        <v>183.5799175357749</v>
+        <v>250.6291390728477</v>
       </c>
       <c r="I66" t="b">
         <v>0</v>
@@ -3353,7 +3353,7 @@
       </c>
       <c r="G67" t="inlineStr"/>
       <c r="H67" t="n">
-        <v>127.4047186932849</v>
+        <v>117.9831932773109</v>
       </c>
       <c r="I67" t="b">
         <v>0</v>
@@ -3398,7 +3398,7 @@
         <v>7.289119583372683</v>
       </c>
       <c r="H68" t="n">
-        <v>125.6394823954258</v>
+        <v>106.1530638189677</v>
       </c>
       <c r="I68" t="b">
         <v>0</v>
@@ -3443,7 +3443,7 @@
         <v>-3.978114349162654</v>
       </c>
       <c r="H69" t="n">
-        <v>203.0436055019022</v>
+        <v>172.2442899702085</v>
       </c>
       <c r="I69" t="b">
         <v>0</v>
@@ -3486,7 +3486,7 @@
       </c>
       <c r="G70" t="inlineStr"/>
       <c r="H70" t="n">
-        <v>180.8968331411337</v>
+        <v>191.1916369773111</v>
       </c>
       <c r="I70" t="b">
         <v>0</v>
@@ -3529,7 +3529,7 @@
       </c>
       <c r="G71" t="inlineStr"/>
       <c r="H71" t="n">
-        <v>234.5534026465028</v>
+        <v>173.8375860317683</v>
       </c>
       <c r="I71" t="b">
         <v>0</v>
@@ -3572,7 +3572,7 @@
       </c>
       <c r="G72" t="inlineStr"/>
       <c r="H72" t="n">
-        <v>-346.2900028320589</v>
+        <v>-369.6761271304939</v>
       </c>
       <c r="I72" t="b">
         <v>1</v>
@@ -3617,7 +3617,7 @@
         <v>10.20304470835676</v>
       </c>
       <c r="H73" t="n">
-        <v>138.0638621388748</v>
+        <v>155.9244419004007</v>
       </c>
       <c r="I73" t="b">
         <v>0</v>
@@ -3660,7 +3660,7 @@
       </c>
       <c r="G74" t="inlineStr"/>
       <c r="H74" t="n">
-        <v>-192.218782249742</v>
+        <v>-305.1108441629355</v>
       </c>
       <c r="I74" t="b">
         <v>1</v>
@@ -3703,7 +3703,7 @@
       </c>
       <c r="G75" t="inlineStr"/>
       <c r="H75" t="n">
-        <v>237.3345213849287</v>
+        <v>239.4528992486997</v>
       </c>
       <c r="I75" t="b">
         <v>0</v>
@@ -3746,7 +3746,7 @@
       </c>
       <c r="G76" t="inlineStr"/>
       <c r="H76" t="n">
-        <v>-387.7930802821633</v>
+        <v>-408.0805938494167</v>
       </c>
       <c r="I76" t="b">
         <v>1</v>
@@ -3791,7 +3791,7 @@
         <v>15.44024389751422</v>
       </c>
       <c r="H77" t="n">
-        <v>198.6314907244092</v>
+        <v>200.946595798532</v>
       </c>
       <c r="I77" t="b">
         <v>0</v>
@@ -3834,7 +3834,7 @@
       </c>
       <c r="G78" t="inlineStr"/>
       <c r="H78" t="n">
-        <v>1207.880547490668</v>
+        <v>1537.592397043295</v>
       </c>
       <c r="I78" t="b">
         <v>0</v>
@@ -3879,7 +3879,7 @@
         <v>-1.755412278125101</v>
       </c>
       <c r="H79" t="n">
-        <v>29.05144975221928</v>
+        <v>31.10593445781746</v>
       </c>
       <c r="I79" t="b">
         <v>0</v>
@@ -3967,7 +3967,7 @@
       </c>
       <c r="G81" t="inlineStr"/>
       <c r="H81" t="n">
-        <v>-328.9718637613709</v>
+        <v>-420.3405865657522</v>
       </c>
       <c r="I81" t="b">
         <v>1</v>
@@ -4057,7 +4057,7 @@
         <v>24.94023133872936</v>
       </c>
       <c r="H83" t="n">
-        <v>109.1571467122425</v>
+        <v>126.2747138397503</v>
       </c>
       <c r="I83" t="b">
         <v>0</v>
@@ -4102,7 +4102,7 @@
         <v>-16.81479293772952</v>
       </c>
       <c r="H84" t="n">
-        <v>165.5555555555555</v>
+        <v>159.4238683127572</v>
       </c>
       <c r="I84" t="b">
         <v>0</v>
@@ -4145,7 +4145,7 @@
       </c>
       <c r="G85" t="inlineStr"/>
       <c r="H85" t="n">
-        <v>200.8368819493731</v>
+        <v>213.5221806520577</v>
       </c>
       <c r="I85" t="b">
         <v>0</v>
@@ -4188,7 +4188,7 @@
       </c>
       <c r="G86" t="inlineStr"/>
       <c r="H86" t="n">
-        <v>286.0776743129684</v>
+        <v>294.2990654205607</v>
       </c>
       <c r="I86" t="b">
         <v>0</v>
@@ -4233,7 +4233,7 @@
         <v>18.48596311592985</v>
       </c>
       <c r="H87" t="n">
-        <v>803.3636723387415</v>
+        <v>-413.4623217922606</v>
       </c>
       <c r="I87" t="b">
         <v>0</v>
@@ -4243,7 +4243,7 @@
       </c>
       <c r="K87" t="inlineStr">
         <is>
-          <t>Excellent</t>
+          <t>Weak</t>
         </is>
       </c>
     </row>
@@ -4258,23 +4258,27 @@
           <t>Information Technology</t>
         </is>
       </c>
-      <c r="C88" t="inlineStr"/>
+      <c r="C88" t="n">
+        <v>0.99</v>
+      </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="E88" t="inlineStr"/>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="E88" t="n">
+        <v>2.528508507926756</v>
+      </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Asset Light</t>
         </is>
       </c>
       <c r="G88" t="n">
         <v>10.04678995232531</v>
       </c>
       <c r="H88" t="n">
-        <v>90.47463575888666</v>
+        <v>96.17996051975098</v>
       </c>
       <c r="I88" t="b">
         <v>0</v>
@@ -4319,7 +4323,7 @@
         <v>32.28517405641733</v>
       </c>
       <c r="H89" t="n">
-        <v>168.9006622516556</v>
+        <v>265.9991656236963</v>
       </c>
       <c r="I89" t="b">
         <v>0</v>
@@ -4364,7 +4368,7 @@
         <v>12.53074535363581</v>
       </c>
       <c r="H90" t="n">
-        <v>52.26641998149861</v>
+        <v>48.48398169336384</v>
       </c>
       <c r="I90" t="b">
         <v>0</v>
@@ -4374,7 +4378,7 @@
       </c>
       <c r="K90" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>Average</t>
         </is>
       </c>
     </row>
@@ -4407,7 +4411,7 @@
       </c>
       <c r="G91" t="inlineStr"/>
       <c r="H91" t="n">
-        <v>175.4027926960258</v>
+        <v>197.2222222222222</v>
       </c>
       <c r="I91" t="b">
         <v>0</v>
@@ -4450,7 +4454,7 @@
       </c>
       <c r="G92" t="inlineStr"/>
       <c r="H92" t="n">
-        <v>74.57158651188503</v>
+        <v>91.3337846987136</v>
       </c>
       <c r="I92" t="b">
         <v>0</v>
@@ -4460,7 +4464,7 @@
       </c>
       <c r="K92" t="inlineStr">
         <is>
-          <t>Average</t>
+          <t>Good</t>
         </is>
       </c>
     </row>
@@ -4493,7 +4497,7 @@
       </c>
       <c r="G93" t="inlineStr"/>
       <c r="H93" t="n">
-        <v>-59.83763132760267</v>
+        <v>-70.43282743114109</v>
       </c>
       <c r="I93" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Sprint 5 Day 32 - Capital Allocation Report completed
</commit_message>
<xml_diff>
--- a/output/cashflow_intelligence.xlsx
+++ b/output/cashflow_intelligence.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="CashFlow" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K93"/>
+  <dimension ref="A1:L93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -472,6 +472,11 @@
           <t>capital_allocation_label</t>
         </is>
       </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>capital_allocation_pattern</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -515,6 +520,11 @@
       <c r="K2" t="inlineStr">
         <is>
           <t>Excellent</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Shareholder Returns</t>
         </is>
       </c>
     </row>
@@ -560,6 +570,11 @@
           <t>Good</t>
         </is>
       </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Shareholder Returns</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -603,6 +618,11 @@
           <t>Good</t>
         </is>
       </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -646,6 +666,11 @@
           <t>Good</t>
         </is>
       </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -689,6 +714,11 @@
           <t>Good</t>
         </is>
       </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Shareholder Returns</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -732,6 +762,11 @@
           <t>Average</t>
         </is>
       </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -775,6 +810,11 @@
           <t>Good</t>
         </is>
       </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -818,6 +858,11 @@
           <t>Good</t>
         </is>
       </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Shareholder Returns</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -861,6 +906,11 @@
       <c r="K10" t="inlineStr">
         <is>
           <t>Excellent</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Shareholder Returns</t>
         </is>
       </c>
     </row>
@@ -906,6 +956,11 @@
           <t>Good</t>
         </is>
       </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>Shareholder Returns</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -949,6 +1004,11 @@
           <t>Weak</t>
         </is>
       </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -992,6 +1052,11 @@
       <c r="K13" t="inlineStr">
         <is>
           <t>Good</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -1037,6 +1102,11 @@
           <t>Weak</t>
         </is>
       </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1080,6 +1150,11 @@
       <c r="K15" t="inlineStr">
         <is>
           <t>Average</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -1125,6 +1200,11 @@
           <t>Weak</t>
         </is>
       </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1168,6 +1248,11 @@
           <t>Weak</t>
         </is>
       </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1211,6 +1296,11 @@
           <t>Good</t>
         </is>
       </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>Shareholder Returns</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1254,6 +1344,11 @@
       <c r="K19" t="inlineStr">
         <is>
           <t>Excellent</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>Shareholder Returns</t>
         </is>
       </c>
     </row>
@@ -1299,6 +1394,11 @@
           <t>Weak</t>
         </is>
       </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>Distress Signal</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1344,6 +1444,11 @@
           <t>Good</t>
         </is>
       </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1389,6 +1494,11 @@
           <t>Excellent</t>
         </is>
       </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>Shareholder Returns</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1434,6 +1544,11 @@
           <t>Excellent</t>
         </is>
       </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1477,6 +1592,11 @@
       <c r="K24" t="inlineStr">
         <is>
           <t>Average</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -1522,6 +1642,11 @@
           <t>Weak</t>
         </is>
       </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1565,6 +1690,11 @@
           <t>Good</t>
         </is>
       </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1610,6 +1740,11 @@
           <t>Average</t>
         </is>
       </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1655,6 +1790,11 @@
           <t>Good</t>
         </is>
       </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>Shareholder Returns</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1700,6 +1840,11 @@
           <t>Good</t>
         </is>
       </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1743,6 +1888,11 @@
       <c r="K30" t="inlineStr">
         <is>
           <t>Average</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -1788,6 +1938,11 @@
           <t>Good</t>
         </is>
       </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>Shareholder Returns</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1831,6 +1986,11 @@
           <t>Good</t>
         </is>
       </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1874,6 +2034,11 @@
           <t>Good</t>
         </is>
       </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1917,6 +2082,11 @@
           <t>Good</t>
         </is>
       </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>Shareholder Returns</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1960,6 +2130,11 @@
           <t>Weak</t>
         </is>
       </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2003,6 +2178,11 @@
           <t>Weak</t>
         </is>
       </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2048,6 +2228,11 @@
           <t>Average</t>
         </is>
       </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>Shareholder Returns</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2093,6 +2278,11 @@
           <t>Average</t>
         </is>
       </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>Shareholder Returns</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2136,6 +2326,11 @@
       <c r="K39" t="inlineStr">
         <is>
           <t>Excellent</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>Shareholder Returns</t>
         </is>
       </c>
     </row>
@@ -2181,6 +2376,11 @@
           <t>Weak</t>
         </is>
       </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2224,6 +2424,11 @@
           <t>Good</t>
         </is>
       </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>Shareholder Returns</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2267,6 +2472,11 @@
       <c r="K42" t="inlineStr">
         <is>
           <t>Good</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>Shareholder Returns</t>
         </is>
       </c>
     </row>
@@ -2312,6 +2522,11 @@
           <t>Good</t>
         </is>
       </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>Shareholder Returns</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2355,6 +2570,11 @@
       <c r="K44" t="inlineStr">
         <is>
           <t>Good</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>Shareholder Returns</t>
         </is>
       </c>
     </row>
@@ -2400,6 +2620,11 @@
           <t>Good</t>
         </is>
       </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2443,6 +2668,11 @@
       <c r="K46" t="inlineStr">
         <is>
           <t>Excellent</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>Shareholder Returns</t>
         </is>
       </c>
     </row>
@@ -2488,6 +2718,11 @@
           <t>Weak</t>
         </is>
       </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>Unclassified</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2531,6 +2766,11 @@
           <t>Good</t>
         </is>
       </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>Shareholder Returns</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2574,6 +2814,11 @@
           <t>Weak</t>
         </is>
       </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>Pre-Revenue</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2619,6 +2864,11 @@
           <t>Good</t>
         </is>
       </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2664,6 +2914,11 @@
           <t>Excellent</t>
         </is>
       </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>Shareholder Returns</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2707,6 +2962,11 @@
       <c r="K52" t="inlineStr">
         <is>
           <t>Good</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -2752,6 +3012,11 @@
           <t>Good</t>
         </is>
       </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>Shareholder Returns</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2795,6 +3060,11 @@
       <c r="K54" t="inlineStr">
         <is>
           <t>Excellent</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
         </is>
       </c>
     </row>
@@ -2840,6 +3110,11 @@
           <t>Good</t>
         </is>
       </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -2883,6 +3158,11 @@
       <c r="K56" t="inlineStr">
         <is>
           <t>Weak</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>Unclassified</t>
         </is>
       </c>
     </row>
@@ -2928,6 +3208,11 @@
           <t>Good</t>
         </is>
       </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -2971,6 +3256,11 @@
           <t>Good</t>
         </is>
       </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>Shareholder Returns</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -3014,6 +3304,11 @@
           <t>Good</t>
         </is>
       </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -3057,6 +3352,11 @@
       <c r="K60" t="inlineStr">
         <is>
           <t>Average</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -3102,6 +3402,11 @@
           <t>Good</t>
         </is>
       </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -3145,6 +3450,11 @@
           <t>Good</t>
         </is>
       </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -3188,6 +3498,11 @@
       <c r="K63" t="inlineStr">
         <is>
           <t>Good</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>Shareholder Returns</t>
         </is>
       </c>
     </row>
@@ -3233,6 +3548,11 @@
           <t>Weak</t>
         </is>
       </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -3278,6 +3598,11 @@
           <t>Excellent</t>
         </is>
       </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>Shareholder Returns</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -3321,6 +3646,11 @@
       <c r="K66" t="inlineStr">
         <is>
           <t>Average</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -3366,6 +3696,11 @@
           <t>Good</t>
         </is>
       </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -3411,6 +3746,11 @@
           <t>Average</t>
         </is>
       </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>Shareholder Returns</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -3454,6 +3794,11 @@
       <c r="K69" t="inlineStr">
         <is>
           <t>Average</t>
+        </is>
+      </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>Shareholder Returns</t>
         </is>
       </c>
     </row>
@@ -3499,6 +3844,11 @@
           <t>Good</t>
         </is>
       </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>Shareholder Returns</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -3542,6 +3892,11 @@
           <t>Good</t>
         </is>
       </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>Shareholder Returns</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -3585,6 +3940,11 @@
           <t>Weak</t>
         </is>
       </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -3628,6 +3988,11 @@
       <c r="K73" t="inlineStr">
         <is>
           <t>Good</t>
+        </is>
+      </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>Shareholder Returns</t>
         </is>
       </c>
     </row>
@@ -3673,6 +4038,11 @@
           <t>Weak</t>
         </is>
       </c>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -3716,6 +4086,11 @@
           <t>Good</t>
         </is>
       </c>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t>Shareholder Returns</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -3759,6 +4134,11 @@
           <t>Weak</t>
         </is>
       </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -3802,6 +4182,11 @@
       <c r="K77" t="inlineStr">
         <is>
           <t>Excellent</t>
+        </is>
+      </c>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t>Shareholder Returns</t>
         </is>
       </c>
     </row>
@@ -3847,6 +4232,11 @@
           <t>Good</t>
         </is>
       </c>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t>Shareholder Returns</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -3892,6 +4282,11 @@
           <t>Average</t>
         </is>
       </c>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -3935,6 +4330,11 @@
       <c r="K80" t="inlineStr">
         <is>
           <t>Average</t>
+        </is>
+      </c>
+      <c r="L80" t="inlineStr">
+        <is>
+          <t>Shareholder Returns</t>
         </is>
       </c>
     </row>
@@ -3980,6 +4380,11 @@
           <t>Weak</t>
         </is>
       </c>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -4025,6 +4430,11 @@
           <t>Good</t>
         </is>
       </c>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -4070,6 +4480,11 @@
           <t>Excellent</t>
         </is>
       </c>
+      <c r="L83" t="inlineStr">
+        <is>
+          <t>Shareholder Returns</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -4113,6 +4528,11 @@
       <c r="K84" t="inlineStr">
         <is>
           <t>Average</t>
+        </is>
+      </c>
+      <c r="L84" t="inlineStr">
+        <is>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -4158,6 +4578,11 @@
           <t>Good</t>
         </is>
       </c>
+      <c r="L85" t="inlineStr">
+        <is>
+          <t>Shareholder Returns</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -4201,6 +4626,11 @@
           <t>Good</t>
         </is>
       </c>
+      <c r="L86" t="inlineStr">
+        <is>
+          <t>Shareholder Returns</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -4246,6 +4676,11 @@
           <t>Weak</t>
         </is>
       </c>
+      <c r="L87" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -4291,6 +4726,11 @@
           <t>Good</t>
         </is>
       </c>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -4336,6 +4776,11 @@
           <t>Excellent</t>
         </is>
       </c>
+      <c r="L89" t="inlineStr">
+        <is>
+          <t>Shareholder Returns</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -4379,6 +4824,11 @@
       <c r="K90" t="inlineStr">
         <is>
           <t>Average</t>
+        </is>
+      </c>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -4424,6 +4874,11 @@
           <t>Good</t>
         </is>
       </c>
+      <c r="L91" t="inlineStr">
+        <is>
+          <t>Shareholder Returns</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -4467,6 +4922,11 @@
           <t>Good</t>
         </is>
       </c>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -4508,6 +4968,11 @@
       <c r="K93" t="inlineStr">
         <is>
           <t>Weak</t>
+        </is>
+      </c>
+      <c r="L93" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
         </is>
       </c>
     </row>

</xml_diff>